<commit_message>
#14 All changes updated in PCB and deliverables and BOM generated
</commit_message>
<xml_diff>
--- a/Design Files/Smart-Power-Supply-v4.0.0/BOM/Client-BOM-Smart Power Supply Unit-v4.0.0.xlsx
+++ b/Design Files/Smart-Power-Supply-v4.0.0/BOM/Client-BOM-Smart Power Supply Unit-v4.0.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12330"/>
+    <workbookView windowWidth="19635" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="86">
   <si>
     <t>#</t>
   </si>
@@ -37,13 +37,13 @@
     <t>Manufacturer</t>
   </si>
   <si>
-    <t>Value</t>
+    <t>Comment</t>
   </si>
   <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>Remarks</t>
+    <t xml:space="preserve"> Remarks</t>
   </si>
   <si>
     <t>Capacitor</t>
@@ -85,9 +85,6 @@
     <t>JSMSEMI</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>FFC/FPC Connector</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
     <t>CONN FFC BOTTOM 30POS 0.5MM R/A</t>
   </si>
   <si>
-    <t>Custom</t>
-  </si>
-  <si>
     <t>FH12-30S-0.5SH(55)</t>
   </si>
   <si>
@@ -112,28 +106,40 @@
     <t>LED1</t>
   </si>
   <si>
-    <t>20mA  67mcd~195mcd -30℃~+85℃ 615nm~630nm  Red 130° 65mW 1.6V~2.6V 0805 Light Emitting Diodes (LED) ROHS</t>
-  </si>
-  <si>
-    <t>LED-0805</t>
-  </si>
-  <si>
-    <t>NCD0805R1</t>
+    <t>10mA 无色透明透镜 80mcd~220mcd 463nm~475nm -30℃~+85℃ Blue 130° 72mW 2.6V~3.6V 0603 Light Emitting Diodes (LED) ROHS</t>
+  </si>
+  <si>
+    <t>LED-0603</t>
+  </si>
+  <si>
+    <t>NCD0603B1</t>
   </si>
   <si>
     <t>Foshan NationStar Optoelectronics</t>
   </si>
   <si>
+    <t>BLUE</t>
+  </si>
+  <si>
     <t>LED2, LED3, LED4, LED5</t>
   </si>
   <si>
-    <t>LED CLA1B-WKW/MKW COOL WHT 4PLCC</t>
-  </si>
-  <si>
-    <t>CLA1B-WKW-XD0F0E33</t>
-  </si>
-  <si>
-    <t>Cree</t>
+    <t>5mA 200mcd~300mcd 雾状黄透镜 -30℃~+85℃ White 130° 72mW 2.6V~3.6V 0603 Light Emitting Diodes (LED) ROHS</t>
+  </si>
+  <si>
+    <t>NCD0603W1</t>
+  </si>
+  <si>
+    <t>WHITE</t>
+  </si>
+  <si>
+    <t>P10, P11, P14, P15</t>
+  </si>
+  <si>
+    <t>WIREPAD</t>
+  </si>
+  <si>
+    <t>Wirepad</t>
   </si>
   <si>
     <t>MOSFET</t>
@@ -172,7 +178,7 @@
     <t>Resistor</t>
   </si>
   <si>
-    <t>R1, R2, R6</t>
+    <t>R1, R2, R6, R11</t>
   </si>
   <si>
     <t>RES 100K OHM 5% 1/10W 0603</t>
@@ -187,7 +193,7 @@
     <t>100K</t>
   </si>
   <si>
-    <t>R3, R5, R12</t>
+    <t>R3, R5, R12, R13</t>
   </si>
   <si>
     <t>RES SMD 4.7K OHM 1% 1/10W 0603</t>
@@ -199,31 +205,40 @@
     <t>4.7K</t>
   </si>
   <si>
-    <t>R4, R7, R8, R9, R10</t>
-  </si>
-  <si>
-    <t>RES SMD 200 OHM 1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>AC0603FR-07200RL</t>
-  </si>
-  <si>
-    <t>200R</t>
-  </si>
-  <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>100mW ±5% 10kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
-  </si>
-  <si>
-    <t>RMC060310K5%N</t>
-  </si>
-  <si>
-    <t>TyoHM</t>
-  </si>
-  <si>
-    <t>10k</t>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>100mW Thick Film Resistors 75V ±100ppm/℃ ±1% 1kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>RC0603FR-071KL</t>
+  </si>
+  <si>
+    <t>YAGEO</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>R7, R8, R9, R10</t>
+  </si>
+  <si>
+    <t>100mW Thick Film Resistors ±100ppm/℃ ±1% 20Ω 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>0603WAF200JT5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(Uniroyal Elec)</t>
+  </si>
+  <si>
+    <t>20R</t>
+  </si>
+  <si>
+    <t>R14</t>
+  </si>
+  <si>
+    <t>DNP</t>
   </si>
   <si>
     <t>Switch</t>
@@ -264,12 +279,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,8 +328,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -464,7 +485,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -485,6 +506,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF03A4CB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -670,7 +697,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -757,6 +784,68 @@
         <color auto="1"/>
       </top>
       <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -862,70 +951,67 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -940,74 +1026,77 @@
     <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1044,11 +1133,49 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1375,7 +1502,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -1399,11 +1526,11 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
-    <row r="2" ht="15.75" spans="1:11">
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1493,7 +1620,7 @@
         <v>22</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J4" s="12">
         <v>1</v>
@@ -1507,25 +1634,25 @@
         <v>3</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>29</v>
-      </c>
       <c r="I5" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J5" s="9">
         <v>1</v>
@@ -1539,318 +1666,396 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="G6" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="H6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="I6" s="13" t="s">
         <v>34</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>23</v>
       </c>
       <c r="J6" s="12">
         <v>1</v>
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="24.75" spans="1:11">
+    <row r="7" ht="36.75" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f>ROW(B7)-ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="F7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="G7" s="10" t="s">
+      <c r="H7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>23</v>
       </c>
       <c r="J7" s="9">
         <v>4</v>
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" ht="15.75" spans="1:11">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f t="shared" ref="B8:B15" si="0">ROW(B8)-ROW($B$2)</f>
+        <f>ROW(B8)-ROW($B$2)</f>
         <v>6</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="11"/>
+      <c r="D8" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="G8" s="13"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="J8" s="9">
-        <v>1</v>
-      </c>
-      <c r="K8" s="9"/>
+      <c r="J8" s="12">
+        <v>4</v>
+      </c>
+      <c r="K8" s="12"/>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" ht="15.75" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B9)-ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="12" t="s">
+      <c r="C9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="H9" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" s="12">
-        <v>2</v>
-      </c>
-      <c r="K9" s="12"/>
+      <c r="I9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="9">
+        <v>1</v>
+      </c>
+      <c r="K9" s="9"/>
     </row>
     <row r="10" ht="15.75" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B10)-ROW($B$2)</f>
         <v>8</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="H10" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" s="9">
-        <v>3</v>
-      </c>
-      <c r="K10" s="9"/>
+      <c r="I10" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="J10" s="12">
+        <v>2</v>
+      </c>
+      <c r="K10" s="12"/>
     </row>
     <row r="11" ht="15.75" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B11)-ROW($B$2)</f>
         <v>9</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="H11" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="J11" s="12">
-        <v>3</v>
-      </c>
-      <c r="K11" s="12"/>
+      <c r="J11" s="9">
+        <v>4</v>
+      </c>
+      <c r="K11" s="9"/>
     </row>
     <row r="12" ht="15.75" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B12)-ROW($B$2)</f>
         <v>10</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="C12" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="H12" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="J12" s="9">
-        <v>5</v>
-      </c>
-      <c r="K12" s="9"/>
+      <c r="J12" s="12">
+        <v>4</v>
+      </c>
+      <c r="K12" s="12"/>
     </row>
-    <row r="13" ht="24.75" spans="1:11">
+    <row r="13" ht="36.75" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B13)-ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="H13" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="G13" s="13" t="s">
+      <c r="I13" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="I13" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="J13" s="12">
+      <c r="J13" s="9">
         <v>1</v>
       </c>
-      <c r="K13" s="12"/>
+      <c r="K13" s="9"/>
     </row>
     <row r="14" ht="36.75" spans="1:11">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B14)-ROW($B$2)</f>
         <v>12</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="H14" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="I14" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="J14" s="9">
-        <v>2</v>
-      </c>
-      <c r="K14" s="9"/>
+      <c r="J14" s="12">
+        <v>4</v>
+      </c>
+      <c r="K14" s="12"/>
     </row>
     <row r="15" ht="15.75" spans="1:11">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f t="shared" si="0"/>
+        <f>ROW(B15)-ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="J15" s="9">
+        <v>1</v>
+      </c>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" ht="36.75" spans="1:11">
+      <c r="A16" s="2"/>
+      <c r="B16" s="7">
+        <f>ROW(B16)-ROW($B$2)</f>
+        <v>14</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D16" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E16" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F16" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G16" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="H15" s="12" t="s">
+      <c r="I16" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="J16" s="12">
+        <v>2</v>
+      </c>
+      <c r="K16" s="12"/>
+    </row>
+    <row r="17" ht="15.75" spans="1:11">
+      <c r="A17" s="2"/>
+      <c r="B17" s="7">
+        <f>ROW(B17)-ROW($B$2)</f>
+        <v>15</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="I15" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="J15" s="12">
+      <c r="D17" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J17" s="9">
         <v>1</v>
       </c>
-      <c r="K15" s="12"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="2"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="25"/>
+    </row>
+    <row r="19" ht="15.75" spans="1:11">
+      <c r="A19" s="2"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>